<commit_message>
Updated website and data
</commit_message>
<xml_diff>
--- a/data/Data.xlsx
+++ b/data/Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Web Development\Indian Against India\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06EE9866-865F-49DF-9075-20FADE522E32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB70E153-F9DB-4F76-AB73-986B30D1CB7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
   <si>
     <t>Year</t>
   </si>
@@ -259,9 +259,6 @@
     <t>Congress, CPI(M), CPI, NC, PDP, TMC, DMK, AAP, SP, RJD, People's Union for Civil Liberties, Foreign-funded Activist NGOs</t>
   </si>
   <si>
-    <t>Congress, CPI(M), CPI, TMC, DMK, AAP, activist NGOs, Foreign-funded Activist NGOs</t>
-  </si>
-  <si>
     <t>Congress, CPI(M), CPI, TMC, AAP, DMK, RJD, SP, NCP, Shiv Sena (UBT), Foreign-funded Activist NGOs, Pseudo-Environmentalist</t>
   </si>
   <si>
@@ -394,6 +391,75 @@
   </si>
   <si>
     <t>https://www.indiatoday.in/news-analysis/story/a-tale-of-u-turns-on-the-three-farm-laws-1750146-2020-12-16</t>
+  </si>
+  <si>
+    <t>Kudankulam Nuclear Power Plant (Tamil Nadu)</t>
+  </si>
+  <si>
+    <t>Kudankulam is the beating heart of India’s energy security and strategic sovereignty. As India’s largest nuclear power station, it crushes our reliance on imported fossil fuels and hostile geopolitical energy blackmail. Generating gigawatts of unceasing, clean baseload power, it single-handedly fuels the massive industrial corridors of Southern India, powering defense manufacturing and high-tech infrastructure critical for national survival. It represents a monumental triumph of indigenous integration and strategic Indo-Russian partnership, built to survive the harshest extremes. In a world where energy starvation is weaponized to cripple sovereign nations, Kudankulam is an impregnable fortress of Atmanirbhar power—ensuring the Indian military-industrial complex and the economic engine of 1.4 billion citizens never go dark.</t>
+  </si>
+  <si>
+    <t>Congress, CPI(M), CPI, TMC, DMK, AAP,  Foreign-funded Activist NGOs</t>
+  </si>
+  <si>
+    <t>Anti-nuclear activists and foreign-funded NGOs flooded the Madras High Court and Supreme Court with PILs. Weaponizing the Fukushima disaster, they demanded a permanent halt to the project. They manufactured panic over environmental clearances, coastal regulation zone norms, nuclear liability, and disaster management, attempting to trap the critical strategic asset in endless judicial paralysis.</t>
+  </si>
+  <si>
+    <t>National security and scientific truth decimated the obstructionists. In May 2013, the Supreme Court unequivocally greenlit the project, ruling that nuclear energy is a vital sovereign necessity for economic growth and national security. Units 1 and 2 were successfully commissioned, and further reactors are rapidly advancing toward integration.</t>
+  </si>
+  <si>
+    <t>Vicious street blockades, orchestrated hunger strikes by the People's Movement Against Nuclear Energy (PMANE), and relentless legal sabotage halted construction and commissioning of Unit 1 for several critical years, pushing its grid synchronization from 2011 to 2013 and bleeding vast amounts of public funds.</t>
+  </si>
+  <si>
+    <t>The vicious campaign engineered by the Congress, the Left parties, DMK, and their INDI alliance ecosystem to choke the Kudankulam project was an egregious assault on India's national security and economic sovereignty. While foreign powers rapidly expanded their nuclear footprints to dominate the geopolitical energy grid, these regressive political outfits actively provided cover to foreign-funded NGOs and radical anarchists to paralyze a multi-billion-dollar strategic asset.
+By blockading the plant and fear-mongering among local populations, they deliberately starved Southern India of critical baseload electricity, crippling industrial output and causing thousands of crores in cost overruns for the national exchequer. Most unforgivably, their anti-development obstructionism directly compromised India's internal security. The then-Prime Minister Manmohan Singh himself admitted that foreign-funded NGOs were funneling dark money to stall the project, yet the broader opposition ecosystem unabashedly backed the agitators to score cheap vote-bank points.
+Every day Kudankulam was delayed, India was forced to rely on imported coal and foreign oil, bleeding foreign exchange and leaving our strategic defense manufacturing vulnerable to power deficits. Sacrificing India's self-reliance in advanced nuclear technology on the altar of foreign-funded activism and cynical electoral opportunism proves these opposition forces are fundamentally hostile to India's rise as an independent, unshakeable global superpower.</t>
+  </si>
+  <si>
+    <t>https://www.ndtv.com/india-news/kudankulam-protesters-getting-support-from-foreign-ngos-govt-498955</t>
+  </si>
+  <si>
+    <t>https://www.hindustantimes.com/delhi/3-ngos-diverted-foreign-funds-to-fuel-kudankulam-stir/story-iI1kYENA42b8JDolIrFkUI.html</t>
+  </si>
+  <si>
+    <t>https://www.businesstoday.in/industry/energy/story/sc-dismisses-plea-against-kudankulam-nuclear-power-plant-41070-2013-05-06</t>
+  </si>
+  <si>
+    <t>https://www.indiatoday.in/india/south/story/v-s-achuthanandan-stopped-from-visiting-kundankulam-116313-2012-09-17</t>
+  </si>
+  <si>
+    <t>POSCO $12 Billion Mega Steel Plant (Odisha)</t>
+  </si>
+  <si>
+    <t>The POSCO mega steel plant was an unprecedented $12 billion Foreign Direct Investment—the largest in India’s history at the time—designed to produce 12 million tonnes of high-grade steel annually. This was a monumental strategic asset for India's infrastructure and defense sovereignty. Domestic production of high-tensile steel is the backbone of naval shipbuilding, armored combat vehicles, and critical border infrastructure. Coupled with a captive deep-sea port at Jatadhar, this project was poised to shatter reliance on foreign supply chains, integrate India into global manufacturing networks, and permanently transform Odisha’s economy by creating tens of thousands of direct and indirect industrial jobs. It represented a crucial leap toward absolute self-reliance and geopolitical strength in strategic heavy manufacturing.</t>
+  </si>
+  <si>
+    <t>Congress, CPI(M), CPI, DMK, AAP, MDMK, PMANE, Foreign-Funded Activist NGOs, Pseudo-Environmentalist</t>
+  </si>
+  <si>
+    <t>Congress, CPI(M), CPI, POSCO Pratirodh Sangram Samiti (PPSS), Local Activist Groups, Foreign-Funded Activist NGOs</t>
+  </si>
+  <si>
+    <t>The project faced a relentless barrage of litigation before the National Green Tribunal (NGT), the Orissa High Court, and the Supreme Court. Opponents weaponized the Forest Rights Act (FRA) and Coastal Regulation Zone (CRZ) norms to file endless petitions, successfully forcing temporary suspensions of environmental clearances and trapping the land acquisition process in insurmountable judicial and bureaucratic gridlock.</t>
+  </si>
+  <si>
+    <t>After 12 years of extreme regulatory hurdles, violent ground protests, and shifting policies regarding captive iron ore mine allocations, POSCO officially withdrew from the project in 2017. The South Korean giant surrendered the acquired land, officially terminating India's largest-ever FDI initiative.</t>
+  </si>
+  <si>
+    <t>The project was completely paralyzed from the signing of the MoU in 2005 until its ultimate cancellation in 2017. Twelve years of land acquisition blockades, procedural delays, and legal injunctions prevented the massive manufacturing facility from ever being constructed.</t>
+  </si>
+  <si>
+    <t>The collapse of the POSCO mega steel plant stands as a colossal failure of India’s industrial ambitions and a severe, self-inflicted blow to its strategic economic sovereignty. While global competitors rapidly expanded their steel dominance and military-industrial capacities, India allowed a transformative $12 billion strategic investment to be systematically dismantled by endless protests, political obstructionism, and regulatory paralysis.
+By driving away this massive facility, India was deprived of 12 million tonnes of domestic high-grade steel production, which is absolutely essential for heavy infrastructure, rapid defense modernization, and naval expansion. The failure fractured global investor confidence, sending a damaging signal to international partners that critical infrastructure projects in India could be indefinitely stalled by political agitations and bureaucratic red tape. Furthermore, it robbed the state of Odisha of massive sovereign revenue and destroyed the prospect of tens of thousands of high-paying jobs for impoverished youth. The relentless opposition and subsequent withdrawal of POSCO severely hampered India's trajectory toward becoming a self-reliant global manufacturing superpower, forcing continued reliance on external supply chains and allowing hostile geopolitical rivals to maintain their dominance in strategic material production.</t>
+  </si>
+  <si>
+    <t>https://www.livemint.com/Companies/1r9u9TWe7q554c8xJFwwlM/Posco-said-to-be-backing-away-from-12-billion-India-project.html</t>
+  </si>
+  <si>
+    <t>https://economictimes.indiatimes.com/industry/indl-goods/svs/steel/south-koreas-posco-suspends-planned-12-bn-odisha-steel-project/articleshow/48101950.cms?from=mdr</t>
+  </si>
+  <si>
+    <t>https://www.business-humanrights.org/en/latest-news/india-amid-resistance-from-communities-posco-offers-to-surrender-land-acquired-for-12-billion-steel-project/</t>
   </si>
 </sst>
 </file>
@@ -514,8 +580,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2DB3396E-FD0B-4F9C-842A-9832690A92E5}" name="Table2" displayName="Table2" ref="A1:L11" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
-  <autoFilter ref="A1:L11" xr:uid="{2DB3396E-FD0B-4F9C-842A-9832690A92E5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2DB3396E-FD0B-4F9C-842A-9832690A92E5}" name="Table2" displayName="Table2" ref="A1:L13" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="A1:L13" xr:uid="{2DB3396E-FD0B-4F9C-842A-9832690A92E5}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L11">
     <sortCondition ref="A1:A11"/>
   </sortState>
@@ -823,7 +889,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B667CDE-8E2B-439F-AECC-B04A1264504F}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -957,37 +1023,37 @@
         <v>2016</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="L4" s="3" t="s">
         <v>107</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="409.5" x14ac:dyDescent="0.25">
@@ -1039,7 +1105,7 @@
         <v>41</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>42</v>
@@ -1077,7 +1143,7 @@
         <v>31</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>32</v>
@@ -1109,34 +1175,34 @@
         <v>2020</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="I8" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="J8" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="K8" s="3" t="s">
         <v>117</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>118</v>
       </c>
       <c r="L8" s="2"/>
     </row>
@@ -1145,34 +1211,34 @@
         <v>2022</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="I9" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="J9" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="J9" s="3" t="s">
+      <c r="K9" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>97</v>
       </c>
       <c r="L9" s="2"/>
     </row>
@@ -1181,37 +1247,37 @@
         <v>2024</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="D10" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="I10" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="L10" s="3" t="s">
         <v>83</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="330" x14ac:dyDescent="0.25">
@@ -1225,7 +1291,7 @@
         <v>46</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>74</v>
+        <v>120</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>47</v>
@@ -1249,6 +1315,80 @@
         <v>26</v>
       </c>
       <c r="L11" s="2"/>
+    </row>
+    <row r="12" spans="1:12" ht="390" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>2001</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="345" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>2005</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="L13" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1289,10 +1429,17 @@
     <hyperlink ref="I8" r:id="rId35" xr:uid="{927FA52B-EC13-4B9D-A3FD-27852A689C4B}"/>
     <hyperlink ref="J8" r:id="rId36" xr:uid="{5DD038AE-667D-4FA2-958D-B30E95434B80}"/>
     <hyperlink ref="K8" r:id="rId37" xr:uid="{43BF0A6D-76E3-484A-8993-305D643EA8F4}"/>
+    <hyperlink ref="I12" r:id="rId38" xr:uid="{0231CA09-72F3-4265-BE34-0B50995AF7B8}"/>
+    <hyperlink ref="J12" r:id="rId39" xr:uid="{E0679219-1095-4E52-A071-57264531CE9A}"/>
+    <hyperlink ref="K12" r:id="rId40" xr:uid="{32EE5611-1A29-45F6-B740-D210D9DF256F}"/>
+    <hyperlink ref="L12" r:id="rId41" xr:uid="{60061CF6-3F99-44AD-85D9-2D58C431A35E}"/>
+    <hyperlink ref="I13" r:id="rId42" xr:uid="{F201AD63-64AB-4E23-B1A2-A754D95D05BB}"/>
+    <hyperlink ref="J13" r:id="rId43" xr:uid="{C5EB7AEA-82C5-46D6-A06A-72D974C5ACD3}"/>
+    <hyperlink ref="K13" r:id="rId44" xr:uid="{0247CA60-0A5B-4BF2-9011-61F24CD43C64}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId38"/>
+    <tablePart r:id="rId45"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>